<commit_message>
Update ASel value for B-type and lui
</commit_message>
<xml_diff>
--- a/proj3/cpu/ROM Control Logic_Truth Table.xlsx
+++ b/proj3/cpu/ROM Control Logic_Truth Table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/terrysmac/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/terrysmac/cs61c-self-study/proj3/cpu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3CD5F4B-1892-E541-BC69-475D822DF9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11242CA5-DE52-324B-9460-9565553E2D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25760" yWindow="840" windowWidth="24620" windowHeight="17140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,6 +48,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -107,6 +108,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -123,6 +125,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -139,6 +142,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -647,7 +651,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -728,6 +732,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -914,6 +925,16 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -921,7 +942,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -933,15 +953,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1190,60 +1201,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="27" t="s">
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="29"/>
-      <c r="H1" s="30" t="s">
+      <c r="G1" s="32"/>
+      <c r="H1" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="29"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="32"/>
       <c r="P1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="31" t="s">
+      <c r="Q1" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="R1" s="32"/>
-      <c r="S1" s="32"/>
-      <c r="T1" s="32"/>
-      <c r="U1" s="32"/>
-      <c r="V1" s="32"/>
-      <c r="W1" s="33"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="36"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="26"/>
+      <c r="A2" s="30"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="3"/>
       <c r="F2" s="1"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="34" t="s">
+      <c r="H2" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="29"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="32"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
@@ -1369,10 +1380,10 @@
       <c r="A5" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="25" t="s">
         <v>35</v>
       </c>
       <c r="D5" s="16" t="s">
@@ -1449,8 +1460,8 @@
       <c r="A6" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
       <c r="D6" s="16" t="s">
         <v>36</v>
       </c>
@@ -1525,8 +1536,8 @@
       <c r="A7" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
       <c r="D7" s="16" t="s">
         <v>36</v>
       </c>
@@ -1601,8 +1612,8 @@
       <c r="A8" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
       <c r="D8" s="16" t="s">
         <v>50</v>
       </c>
@@ -1677,8 +1688,8 @@
       <c r="A9" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
       <c r="D9" s="19" t="s">
         <v>50</v>
       </c>
@@ -1753,8 +1764,8 @@
       <c r="A10" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
       <c r="D10" s="16" t="s">
         <v>55</v>
       </c>
@@ -1829,8 +1840,8 @@
       <c r="A11" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
       <c r="D11" s="16" t="s">
         <v>58</v>
       </c>
@@ -1905,8 +1916,8 @@
       <c r="A12" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
       <c r="D12" s="16" t="s">
         <v>61</v>
       </c>
@@ -1981,8 +1992,8 @@
       <c r="A13" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
       <c r="D13" s="16" t="s">
         <v>64</v>
       </c>
@@ -2057,8 +2068,8 @@
       <c r="A14" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
       <c r="D14" s="16" t="s">
         <v>64</v>
       </c>
@@ -2133,8 +2144,8 @@
       <c r="A15" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
       <c r="D15" s="16" t="s">
         <v>69</v>
       </c>
@@ -2209,8 +2220,8 @@
       <c r="A16" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
       <c r="D16" s="16" t="s">
         <v>72</v>
       </c>
@@ -2285,10 +2296,10 @@
       <c r="A17" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="B17" s="36" t="s">
+      <c r="B17" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="C17" s="37" t="s">
+      <c r="C17" s="28" t="s">
         <v>76</v>
       </c>
       <c r="D17" s="16" t="s">
@@ -2363,8 +2374,8 @@
       <c r="A18" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
       <c r="D18" s="19" t="s">
         <v>50</v>
       </c>
@@ -2437,8 +2448,8 @@
       <c r="A19" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
       <c r="D19" s="16" t="s">
         <v>58</v>
       </c>
@@ -2511,8 +2522,8 @@
       <c r="A20" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="37" t="s">
+      <c r="B20" s="26"/>
+      <c r="C20" s="28" t="s">
         <v>81</v>
       </c>
       <c r="D20" s="16" t="s">
@@ -2587,8 +2598,8 @@
       <c r="A21" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
       <c r="D21" s="19" t="s">
         <v>50</v>
       </c>
@@ -2663,8 +2674,8 @@
       <c r="A22" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
       <c r="D22" s="16" t="s">
         <v>58</v>
       </c>
@@ -2737,8 +2748,8 @@
       <c r="A23" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
       <c r="D23" s="19" t="s">
         <v>61</v>
       </c>
@@ -2811,8 +2822,8 @@
       <c r="A24" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="28"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
       <c r="D24" s="16" t="s">
         <v>64</v>
       </c>
@@ -2887,8 +2898,8 @@
       <c r="A25" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
       <c r="D25" s="16" t="s">
         <v>64</v>
       </c>
@@ -2963,8 +2974,8 @@
       <c r="A26" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
       <c r="D26" s="16" t="s">
         <v>69</v>
       </c>
@@ -3037,8 +3048,8 @@
       <c r="A27" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
       <c r="D27" s="16" t="s">
         <v>72</v>
       </c>
@@ -3111,10 +3122,10 @@
       <c r="A28" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B28" s="36" t="s">
+      <c r="B28" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="C28" s="37" t="s">
+      <c r="C28" s="28" t="s">
         <v>91</v>
       </c>
       <c r="D28" s="16" t="s">
@@ -3189,8 +3200,8 @@
       <c r="A29" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
       <c r="D29" s="19" t="s">
         <v>50</v>
       </c>
@@ -3263,8 +3274,8 @@
       <c r="A30" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
       <c r="D30" s="16" t="s">
         <v>58</v>
       </c>
@@ -3337,10 +3348,10 @@
       <c r="A31" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B31" s="36" t="s">
+      <c r="B31" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="37" t="s">
+      <c r="C31" s="28" t="s">
         <v>97</v>
       </c>
       <c r="D31" s="16" t="s">
@@ -3365,7 +3376,7 @@
         <v>40</v>
       </c>
       <c r="K31" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L31" s="18" t="s">
         <v>38</v>
@@ -3381,15 +3392,15 @@
       </c>
       <c r="P31" s="11" t="str">
         <f t="shared" si="1"/>
-        <v>1044</v>
+        <v>1064</v>
       </c>
       <c r="Q31" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>0001000001000100</v>
+        <v>0001000001100100</v>
       </c>
       <c r="R31" s="12" t="str">
         <f t="shared" si="3"/>
-        <v>01000100</v>
+        <v>01100100</v>
       </c>
       <c r="S31" s="12" t="str">
         <f t="shared" si="4"/>
@@ -3397,7 +3408,7 @@
       </c>
       <c r="T31" s="12" t="str">
         <f t="shared" ref="T31:U31" si="32">BIN2HEX(R31,2)</f>
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="U31" s="13" t="str">
         <f t="shared" si="32"/>
@@ -3415,8 +3426,8 @@
       <c r="A32" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
       <c r="D32" s="19" t="s">
         <v>50</v>
       </c>
@@ -3439,7 +3450,7 @@
         <v>40</v>
       </c>
       <c r="K32" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L32" s="18" t="s">
         <v>38</v>
@@ -3455,15 +3466,15 @@
       </c>
       <c r="P32" s="11" t="str">
         <f t="shared" si="1"/>
-        <v>1044</v>
+        <v>1064</v>
       </c>
       <c r="Q32" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>0001000001000100</v>
+        <v>0001000001100100</v>
       </c>
       <c r="R32" s="12" t="str">
         <f t="shared" si="3"/>
-        <v>01000100</v>
+        <v>01100100</v>
       </c>
       <c r="S32" s="12" t="str">
         <f t="shared" si="4"/>
@@ -3471,7 +3482,7 @@
       </c>
       <c r="T32" s="12" t="str">
         <f t="shared" ref="T32:U32" si="33">BIN2HEX(R32,2)</f>
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="U32" s="13" t="str">
         <f t="shared" si="33"/>
@@ -3489,8 +3500,8 @@
       <c r="A33" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
       <c r="D33" s="19" t="s">
         <v>61</v>
       </c>
@@ -3513,7 +3524,7 @@
         <v>40</v>
       </c>
       <c r="K33" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L33" s="18" t="s">
         <v>38</v>
@@ -3529,15 +3540,15 @@
       </c>
       <c r="P33" s="11" t="str">
         <f t="shared" si="1"/>
-        <v>1044</v>
+        <v>1064</v>
       </c>
       <c r="Q33" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>0001000001000100</v>
+        <v>0001000001100100</v>
       </c>
       <c r="R33" s="12" t="str">
         <f t="shared" si="3"/>
-        <v>01000100</v>
+        <v>01100100</v>
       </c>
       <c r="S33" s="12" t="str">
         <f t="shared" si="4"/>
@@ -3545,7 +3556,7 @@
       </c>
       <c r="T33" s="12" t="str">
         <f t="shared" ref="T33:U33" si="34">BIN2HEX(R33,2)</f>
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="U33" s="13" t="str">
         <f t="shared" si="34"/>
@@ -3563,8 +3574,8 @@
       <c r="A34" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B34" s="28"/>
-      <c r="C34" s="28"/>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
       <c r="D34" s="16" t="s">
         <v>64</v>
       </c>
@@ -3587,7 +3598,7 @@
         <v>40</v>
       </c>
       <c r="K34" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L34" s="18" t="s">
         <v>38</v>
@@ -3603,15 +3614,15 @@
       </c>
       <c r="P34" s="11" t="str">
         <f t="shared" si="1"/>
-        <v>1044</v>
+        <v>1064</v>
       </c>
       <c r="Q34" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>0001000001000100</v>
+        <v>0001000001100100</v>
       </c>
       <c r="R34" s="12" t="str">
         <f t="shared" si="3"/>
-        <v>01000100</v>
+        <v>01100100</v>
       </c>
       <c r="S34" s="12" t="str">
         <f t="shared" si="4"/>
@@ -3619,7 +3630,7 @@
       </c>
       <c r="T34" s="12" t="str">
         <f t="shared" ref="T34:U34" si="35">BIN2HEX(R34,2)</f>
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="U34" s="13" t="str">
         <f t="shared" si="35"/>
@@ -3637,8 +3648,8 @@
       <c r="A35" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
+      <c r="B35" s="26"/>
+      <c r="C35" s="26"/>
       <c r="D35" s="16" t="s">
         <v>69</v>
       </c>
@@ -3661,7 +3672,7 @@
         <v>38</v>
       </c>
       <c r="K35" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L35" s="18" t="s">
         <v>38</v>
@@ -3677,15 +3688,15 @@
       </c>
       <c r="P35" s="11" t="str">
         <f t="shared" si="1"/>
-        <v>1054</v>
+        <v>1074</v>
       </c>
       <c r="Q35" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>0001000001010100</v>
+        <v>0001000001110100</v>
       </c>
       <c r="R35" s="12" t="str">
         <f t="shared" si="3"/>
-        <v>01010100</v>
+        <v>01110100</v>
       </c>
       <c r="S35" s="12" t="str">
         <f t="shared" si="4"/>
@@ -3693,7 +3704,7 @@
       </c>
       <c r="T35" s="12" t="str">
         <f t="shared" ref="T35:U35" si="36">BIN2HEX(R35,2)</f>
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="U35" s="13" t="str">
         <f t="shared" si="36"/>
@@ -3711,8 +3722,8 @@
       <c r="A36" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B36" s="28"/>
-      <c r="C36" s="28"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
       <c r="D36" s="16" t="s">
         <v>72</v>
       </c>
@@ -3735,7 +3746,7 @@
         <v>38</v>
       </c>
       <c r="K36" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L36" s="18" t="s">
         <v>38</v>
@@ -3751,15 +3762,15 @@
       </c>
       <c r="P36" s="11" t="str">
         <f t="shared" si="1"/>
-        <v>1054</v>
+        <v>1074</v>
       </c>
       <c r="Q36" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>0001000001010100</v>
+        <v>0001000001110100</v>
       </c>
       <c r="R36" s="12" t="str">
         <f t="shared" si="3"/>
-        <v>01010100</v>
+        <v>01110100</v>
       </c>
       <c r="S36" s="12" t="str">
         <f t="shared" si="4"/>
@@ -3767,7 +3778,7 @@
       </c>
       <c r="T36" s="12" t="str">
         <f t="shared" ref="T36:U36" si="37">BIN2HEX(R36,2)</f>
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="U36" s="13" t="str">
         <f t="shared" si="37"/>
@@ -3785,7 +3796,7 @@
       <c r="A37" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="B37" s="36" t="s">
+      <c r="B37" s="27" t="s">
         <v>105</v>
       </c>
       <c r="C37" s="23" t="s">
@@ -3861,7 +3872,7 @@
       <c r="A38" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="28"/>
+      <c r="B38" s="26"/>
       <c r="C38" s="23" t="s">
         <v>109</v>
       </c>
@@ -3885,7 +3896,7 @@
         <v>40</v>
       </c>
       <c r="K38" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L38" s="18" t="s">
         <v>38</v>
@@ -3901,15 +3912,15 @@
       </c>
       <c r="P38" s="11" t="str">
         <f t="shared" si="1"/>
-        <v>17C7</v>
+        <v>17E7</v>
       </c>
       <c r="Q38" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>0001011111000111</v>
+        <v>0001011111100111</v>
       </c>
       <c r="R38" s="12" t="str">
         <f t="shared" si="3"/>
-        <v>11000111</v>
+        <v>11100111</v>
       </c>
       <c r="S38" s="12" t="str">
         <f t="shared" si="4"/>
@@ -3917,7 +3928,7 @@
       </c>
       <c r="T38" s="12" t="str">
         <f t="shared" ref="T38:U38" si="39">BIN2HEX(R38,2)</f>
-        <v>C7</v>
+        <v>E7</v>
       </c>
       <c r="U38" s="13" t="str">
         <f t="shared" si="39"/>
@@ -5047,6 +5058,12 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:O1"/>
+    <mergeCell ref="Q1:W1"/>
+    <mergeCell ref="H2:O2"/>
     <mergeCell ref="C5:C16"/>
     <mergeCell ref="B31:B36"/>
     <mergeCell ref="B37:B38"/>
@@ -5057,12 +5074,6 @@
     <mergeCell ref="B28:B30"/>
     <mergeCell ref="C28:C30"/>
     <mergeCell ref="C31:C36"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:O1"/>
-    <mergeCell ref="Q1:W1"/>
-    <mergeCell ref="H2:O2"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="A1:A2">

</xml_diff>

<commit_message>
Update control logic for jalr - ASel for jalr udpate to 0
</commit_message>
<xml_diff>
--- a/proj3/cpu/ROM Control Logic_Truth Table.xlsx
+++ b/proj3/cpu/ROM Control Logic_Truth Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/terrysmac/cs61c-self-study/proj3/cpu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11242CA5-DE52-324B-9460-9565553E2D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45DBEAB-6035-9C44-9414-4CBC40589B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25760" yWindow="840" windowWidth="24620" windowHeight="17140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="24620" windowHeight="16900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Control Logic for ROM" sheetId="1" r:id="rId1"/>
@@ -925,16 +925,6 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -942,6 +932,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -953,6 +944,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1201,60 +1201,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="31" t="s">
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="33" t="s">
+      <c r="G1" s="29"/>
+      <c r="H1" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="32"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="29"/>
       <c r="P1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="34" t="s">
+      <c r="Q1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="36"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="32"/>
+      <c r="T1" s="32"/>
+      <c r="U1" s="32"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="33"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="30"/>
+      <c r="A2" s="26"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="3"/>
       <c r="F2" s="1"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="37" t="s">
+      <c r="H2" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="32"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="29"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
@@ -1380,10 +1380,10 @@
       <c r="A5" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="35" t="s">
         <v>35</v>
       </c>
       <c r="D5" s="16" t="s">
@@ -1460,8 +1460,8 @@
       <c r="A6" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
       <c r="D6" s="16" t="s">
         <v>36</v>
       </c>
@@ -1536,8 +1536,8 @@
       <c r="A7" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
       <c r="D7" s="16" t="s">
         <v>36</v>
       </c>
@@ -1612,8 +1612,8 @@
       <c r="A8" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
       <c r="D8" s="16" t="s">
         <v>50</v>
       </c>
@@ -1688,8 +1688,8 @@
       <c r="A9" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
       <c r="D9" s="19" t="s">
         <v>50</v>
       </c>
@@ -1764,8 +1764,8 @@
       <c r="A10" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
       <c r="D10" s="16" t="s">
         <v>55</v>
       </c>
@@ -1840,8 +1840,8 @@
       <c r="A11" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
       <c r="D11" s="16" t="s">
         <v>58</v>
       </c>
@@ -1916,8 +1916,8 @@
       <c r="A12" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
       <c r="D12" s="16" t="s">
         <v>61</v>
       </c>
@@ -1992,8 +1992,8 @@
       <c r="A13" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
       <c r="D13" s="16" t="s">
         <v>64</v>
       </c>
@@ -2068,8 +2068,8 @@
       <c r="A14" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
       <c r="D14" s="16" t="s">
         <v>64</v>
       </c>
@@ -2144,8 +2144,8 @@
       <c r="A15" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
       <c r="D15" s="16" t="s">
         <v>69</v>
       </c>
@@ -2220,8 +2220,8 @@
       <c r="A16" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
       <c r="D16" s="16" t="s">
         <v>72</v>
       </c>
@@ -2296,10 +2296,10 @@
       <c r="A17" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="37" t="s">
         <v>76</v>
       </c>
       <c r="D17" s="16" t="s">
@@ -2374,8 +2374,8 @@
       <c r="A18" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
       <c r="D18" s="19" t="s">
         <v>50</v>
       </c>
@@ -2448,8 +2448,8 @@
       <c r="A19" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
       <c r="D19" s="16" t="s">
         <v>58</v>
       </c>
@@ -2522,8 +2522,8 @@
       <c r="A20" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="28" t="s">
+      <c r="B20" s="28"/>
+      <c r="C20" s="37" t="s">
         <v>81</v>
       </c>
       <c r="D20" s="16" t="s">
@@ -2598,8 +2598,8 @@
       <c r="A21" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
       <c r="D21" s="19" t="s">
         <v>50</v>
       </c>
@@ -2674,8 +2674,8 @@
       <c r="A22" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
       <c r="D22" s="16" t="s">
         <v>58</v>
       </c>
@@ -2748,8 +2748,8 @@
       <c r="A23" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
       <c r="D23" s="19" t="s">
         <v>61</v>
       </c>
@@ -2822,8 +2822,8 @@
       <c r="A24" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
       <c r="D24" s="16" t="s">
         <v>64</v>
       </c>
@@ -2898,8 +2898,8 @@
       <c r="A25" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
       <c r="D25" s="16" t="s">
         <v>64</v>
       </c>
@@ -2974,8 +2974,8 @@
       <c r="A26" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="28"/>
       <c r="D26" s="16" t="s">
         <v>69</v>
       </c>
@@ -3048,8 +3048,8 @@
       <c r="A27" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
       <c r="D27" s="16" t="s">
         <v>72</v>
       </c>
@@ -3122,10 +3122,10 @@
       <c r="A28" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B28" s="27" t="s">
+      <c r="B28" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="37" t="s">
         <v>91</v>
       </c>
       <c r="D28" s="16" t="s">
@@ -3200,8 +3200,8 @@
       <c r="A29" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
       <c r="D29" s="19" t="s">
         <v>50</v>
       </c>
@@ -3274,8 +3274,8 @@
       <c r="A30" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
       <c r="D30" s="16" t="s">
         <v>58</v>
       </c>
@@ -3348,10 +3348,10 @@
       <c r="A31" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="36" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="37" t="s">
         <v>97</v>
       </c>
       <c r="D31" s="16" t="s">
@@ -3426,8 +3426,8 @@
       <c r="A32" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
       <c r="D32" s="19" t="s">
         <v>50</v>
       </c>
@@ -3500,8 +3500,8 @@
       <c r="A33" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
       <c r="D33" s="19" t="s">
         <v>61</v>
       </c>
@@ -3574,8 +3574,8 @@
       <c r="A34" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B34" s="26"/>
-      <c r="C34" s="26"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="28"/>
       <c r="D34" s="16" t="s">
         <v>64</v>
       </c>
@@ -3648,8 +3648,8 @@
       <c r="A35" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="B35" s="26"/>
-      <c r="C35" s="26"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
       <c r="D35" s="16" t="s">
         <v>69</v>
       </c>
@@ -3722,8 +3722,8 @@
       <c r="A36" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B36" s="26"/>
-      <c r="C36" s="26"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
       <c r="D36" s="16" t="s">
         <v>72</v>
       </c>
@@ -3796,7 +3796,7 @@
       <c r="A37" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="B37" s="27" t="s">
+      <c r="B37" s="36" t="s">
         <v>105</v>
       </c>
       <c r="C37" s="23" t="s">
@@ -3872,7 +3872,7 @@
       <c r="A38" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="26"/>
+      <c r="B38" s="28"/>
       <c r="C38" s="23" t="s">
         <v>109</v>
       </c>
@@ -4050,7 +4050,7 @@
         <v>40</v>
       </c>
       <c r="K40" s="18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="L40" s="18" t="s">
         <v>38</v>
@@ -4066,15 +4066,15 @@
       </c>
       <c r="P40" s="11" t="str">
         <f t="shared" si="1"/>
-        <v>2061</v>
+        <v>2041</v>
       </c>
       <c r="Q40" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>0010000001100001</v>
+        <v>0010000001000001</v>
       </c>
       <c r="R40" s="12" t="str">
         <f t="shared" si="3"/>
-        <v>01100001</v>
+        <v>01000001</v>
       </c>
       <c r="S40" s="12" t="str">
         <f t="shared" si="4"/>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="T40" s="12" t="str">
         <f t="shared" ref="T40:U40" si="41">BIN2HEX(R40,2)</f>
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="U40" s="13" t="str">
         <f t="shared" si="41"/>
@@ -5058,12 +5058,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:O1"/>
-    <mergeCell ref="Q1:W1"/>
-    <mergeCell ref="H2:O2"/>
     <mergeCell ref="C5:C16"/>
     <mergeCell ref="B31:B36"/>
     <mergeCell ref="B37:B38"/>
@@ -5074,6 +5068,12 @@
     <mergeCell ref="B28:B30"/>
     <mergeCell ref="C28:C30"/>
     <mergeCell ref="C31:C36"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:O1"/>
+    <mergeCell ref="Q1:W1"/>
+    <mergeCell ref="H2:O2"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="A1:A2">

</xml_diff>